<commit_message>
vault backup: 2026-10-14 14:46:08
</commit_message>
<xml_diff>
--- a/Клиенты/EkspertAgro/Статистика/report_sales_attribution_2026-10-14.xlsx
+++ b/Клиенты/EkspertAgro/Статистика/report_sales_attribution_2026-10-14.xlsx
@@ -63,10 +63,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,13 +432,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,14 +459,14 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. Источник в продаже и первый контакт</t>
+          <t>1. Сколько продаж записано не на тот канал</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Источник в продаже</t>
+          <t>Источник в CRM сейчас</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -475,7 +476,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Из них первый контакт — рекламный звонок (Google Ads / Facebook)</t>
+          <t>Записано верно</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Перенести в рекламу (был рекламный звонок)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Спорные</t>
         </is>
       </c>
     </row>
@@ -489,7 +500,13 @@
         <v>26</v>
       </c>
       <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
         <v>24</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -502,7 +519,13 @@
         <v>25</v>
       </c>
       <c r="C7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D7" t="n">
         <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -515,6 +538,12 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -528,7 +557,13 @@
         <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>10</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -541,130 +576,144 @@
         <v>68</v>
       </c>
       <c r="C10" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+        <v>42</v>
+      </c>
+      <c r="D10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Перенести — в CRM «Телефон» или «Нет метки», но номер раньше звонил из рекламы Google Ads / Facebook. Спорные — в CRM рекламный источник, а первый звонок пришёл из другого рекламного канала. Остальные продажи записаны верно: у Google Ads и Facebook они пришли через сайт с рекламной меткой.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2. Как изменится число продаж по каналам, если записать их на первый рекламный контакт</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Канал</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Сейчас</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Станет</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Изменение</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Телефон (без рекламного звонка)</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>26</v>
-      </c>
-      <c r="C14" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>-24</t>
-        </is>
-      </c>
+      <c r="E14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Нет метки</t>
+          <t>Телефон (без рекламного звонка)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-24</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Нет метки</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>-1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Google Ads</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="B17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>10</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>30</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>+20</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Всего</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B19" t="n">
         <v>68</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C19" t="n">
         <v>68</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Как читать: продажа переносится в рекламный канал, если до неё есть звонок с рекламным UTM, а в CRM стоит «Телефон» или «Нет метки». Совпадение номера и времени — признак, а не доказательство; поэтому список номеров ниже нужен для ручной проверки.</t>
         </is>
@@ -697,52 +746,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Телефон</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Телефон</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Заказ</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Продажа записана (время Варшавы)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Источник в CRM сейчас</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Первый рекламный звонок (время Варшавы)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Канал звонка</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Когда записана продажа</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Через сколько после начала звонка продажа записана в CRM</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Разговор, сек</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Что проверить</t>
         </is>

</xml_diff>